<commit_message>
5 vlan sujungiau per router
</commit_message>
<xml_diff>
--- a/L2B/Adresai.xlsx
+++ b/L2B/Adresai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Desktop\mokslai\semestras 4\komp-tinklai\L2B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FAFB58-8DE2-43D0-B981-6A27DE0DCEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30239802-7DCE-4195-8D0D-021EAF7F1D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20520" yWindow="6585" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mano individualus IP" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
duoti static ipv4 ir excluded
</commit_message>
<xml_diff>
--- a/L2B/Adresai.xlsx
+++ b/L2B/Adresai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Desktop\mokslai\semestras 4\komp-tinklai\L2B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6CEBDA-01AC-4A3E-A118-665BDD4F0FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E9C2F8F-AA58-4C66-BA21-3259269FEB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20265" yWindow="6735" windowWidth="20370" windowHeight="10770" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20520" yWindow="6585" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mano individualus IP" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
pritaikiau dar acl 4 potinkliui
</commit_message>
<xml_diff>
--- a/L2B/Adresai.xlsx
+++ b/L2B/Adresai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Desktop\mokslai\semestras 4\komp-tinklai\L2B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4863725F-7BDB-4A67-B5A9-81F9BBD13972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674B82B8-E473-44F0-8E4D-2B1EECF8CBCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20520" yWindow="6585" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mano individualus IP" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="161">
   <si>
     <t>Individualus ipv4:</t>
   </si>
@@ -510,6 +510,18 @@
   </si>
   <si>
     <t>Router(config-ipv6-acl)# permit ipv6 any any</t>
+  </si>
+  <si>
+    <t>Router(config)# interface g0/0.2</t>
+  </si>
+  <si>
+    <t>Router(config-subif)# ip access-group BLOKAVIMAS_AUDITORIJOMS in</t>
+  </si>
+  <si>
+    <t>Router(config-subif)# ipv6 traffic-filter BLOKAVIMAS_V6 in</t>
+  </si>
+  <si>
+    <t>pritaikau tai vlan 2, 3, 4 ir 8</t>
   </si>
 </sst>
 </file>
@@ -903,14 +915,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="11.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="66.42578125" customWidth="1"/>
     <col min="2" max="2" width="59.140625" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -918,7 +931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -926,44 +939,56 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>148</v>
       </c>
       <c r="B6" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>147</v>
       </c>
       <c r="B7" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>142</v>
       </c>
       <c r="B8" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>143</v>
       </c>
       <c r="B9" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>144</v>
       </c>
@@ -971,7 +996,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>145</v>
       </c>
@@ -979,7 +1004,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>146</v>
       </c>

</xml_diff>